<commit_message>
update perhitungan proyeksi manfaat
</commit_message>
<xml_diff>
--- a/data/file/tabel_tenor_spot_rate.xlsx
+++ b/data/file/tabel_tenor_spot_rate.xlsx
@@ -5,23 +5,34 @@
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="F:\Kerjaan Arya\KKA VAB\Aplikasi\imbalan-pasca-kerja-app\data\file\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Aryax punya\2026\KKA VAB\Aplikasi\imbalan-pasca-kerja-app\data\file\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{9C7C1568-6791-4D02-A91C-AAE7504604C0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D84EBBF8-EAF8-40D5-9D24-1F744FA6DEA5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{13D302E8-A00F-41E5-906F-072FF2494F16}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{13D302E8-A00F-41E5-906F-072FF2494F16}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="191029"/>
+  <calcPr calcId="181029"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
     </ext>
   </extLst>
 </workbook>
+</file>
+
+<file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2" uniqueCount="2">
+  <si>
+    <t>tenor</t>
+  </si>
+  <si>
+    <t>rate</t>
+  </si>
+</sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
@@ -377,502 +388,510 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1D4B26EF-FE81-4E19-AD0A-2E2FC440C7F4}">
-  <dimension ref="A1:B62"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <dimension ref="A1:B63"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A1">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A1" t="s">
         <v>0</v>
       </c>
-      <c r="B1">
-        <v>4.4800000000000004</v>
-      </c>
-    </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="B1" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="2" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A2">
-        <v>0.5</v>
+        <v>0</v>
       </c>
       <c r="B2">
         <v>4.4800000000000004</v>
       </c>
     </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A3">
+        <v>0.5</v>
+      </c>
+      <c r="B3">
+        <v>4.4800000000000004</v>
+      </c>
+    </row>
+    <row r="4" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A4">
         <v>1</v>
-      </c>
-      <c r="B3">
-        <v>4.8099999999999996</v>
-      </c>
-    </row>
-    <row r="4" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A4">
-        <v>1.5</v>
       </c>
       <c r="B4">
         <v>4.8099999999999996</v>
       </c>
     </row>
-    <row r="5" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A5">
+        <v>1.5</v>
+      </c>
+      <c r="B5">
+        <v>4.8099999999999996</v>
+      </c>
+    </row>
+    <row r="6" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A6">
         <v>2</v>
-      </c>
-      <c r="B5">
-        <v>5.0999999999999996</v>
-      </c>
-    </row>
-    <row r="6" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A6">
-        <v>2.5</v>
       </c>
       <c r="B6">
         <v>5.0999999999999996</v>
       </c>
     </row>
-    <row r="7" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A7">
+        <v>2.5</v>
+      </c>
+      <c r="B7">
+        <v>5.0999999999999996</v>
+      </c>
+    </row>
+    <row r="8" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A8">
         <v>3</v>
-      </c>
-      <c r="B7">
-        <v>5.33</v>
-      </c>
-    </row>
-    <row r="8" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A8">
-        <v>3.5</v>
       </c>
       <c r="B8">
         <v>5.33</v>
       </c>
     </row>
-    <row r="9" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A9">
+        <v>3.5</v>
+      </c>
+      <c r="B9">
+        <v>5.33</v>
+      </c>
+    </row>
+    <row r="10" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A10">
         <v>4</v>
-      </c>
-      <c r="B9">
-        <v>5.52</v>
-      </c>
-    </row>
-    <row r="10" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A10">
-        <v>4.5</v>
       </c>
       <c r="B10">
         <v>5.52</v>
       </c>
     </row>
-    <row r="11" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A11">
+        <v>4.5</v>
+      </c>
+      <c r="B11">
+        <v>5.52</v>
+      </c>
+    </row>
+    <row r="12" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A12">
         <v>5</v>
-      </c>
-      <c r="B11">
-        <v>5.67</v>
-      </c>
-    </row>
-    <row r="12" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A12">
-        <v>5.5</v>
       </c>
       <c r="B12">
         <v>5.67</v>
       </c>
     </row>
-    <row r="13" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A13">
+        <v>5.5</v>
+      </c>
+      <c r="B13">
+        <v>5.67</v>
+      </c>
+    </row>
+    <row r="14" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A14">
         <v>6</v>
-      </c>
-      <c r="B13">
-        <v>5.8</v>
-      </c>
-    </row>
-    <row r="14" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A14">
-        <v>6.5</v>
       </c>
       <c r="B14">
         <v>5.8</v>
       </c>
     </row>
-    <row r="15" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A15">
+        <v>6.5</v>
+      </c>
+      <c r="B15">
+        <v>5.8</v>
+      </c>
+    </row>
+    <row r="16" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A16">
         <v>7</v>
-      </c>
-      <c r="B15">
-        <v>5.92</v>
-      </c>
-    </row>
-    <row r="16" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A16">
-        <v>7.5</v>
       </c>
       <c r="B16">
         <v>5.92</v>
       </c>
     </row>
-    <row r="17" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A17">
+        <v>7.5</v>
+      </c>
+      <c r="B17">
+        <v>5.92</v>
+      </c>
+    </row>
+    <row r="18" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A18">
         <v>8</v>
-      </c>
-      <c r="B17">
-        <v>6.01</v>
-      </c>
-    </row>
-    <row r="18" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A18">
-        <v>8.5</v>
       </c>
       <c r="B18">
         <v>6.01</v>
       </c>
     </row>
-    <row r="19" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A19">
+        <v>8.5</v>
+      </c>
+      <c r="B19">
+        <v>6.01</v>
+      </c>
+    </row>
+    <row r="20" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A20">
         <v>9</v>
-      </c>
-      <c r="B19">
-        <v>6.09</v>
-      </c>
-    </row>
-    <row r="20" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A20">
-        <v>9.5</v>
       </c>
       <c r="B20">
         <v>6.09</v>
       </c>
     </row>
-    <row r="21" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A21">
+        <v>9.5</v>
+      </c>
+      <c r="B21">
+        <v>6.09</v>
+      </c>
+    </row>
+    <row r="22" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A22">
         <v>10</v>
-      </c>
-      <c r="B21">
-        <v>6.16</v>
-      </c>
-    </row>
-    <row r="22" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A22">
-        <v>10.5</v>
       </c>
       <c r="B22">
         <v>6.16</v>
       </c>
     </row>
-    <row r="23" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A23">
+        <v>10.5</v>
+      </c>
+      <c r="B23">
+        <v>6.16</v>
+      </c>
+    </row>
+    <row r="24" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A24">
         <v>11</v>
-      </c>
-      <c r="B23">
-        <v>6.23</v>
-      </c>
-    </row>
-    <row r="24" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A24">
-        <v>11.5</v>
       </c>
       <c r="B24">
         <v>6.23</v>
       </c>
     </row>
-    <row r="25" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A25">
+        <v>11.5</v>
+      </c>
+      <c r="B25">
+        <v>6.23</v>
+      </c>
+    </row>
+    <row r="26" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A26">
         <v>12</v>
-      </c>
-      <c r="B25">
-        <v>6.28</v>
-      </c>
-    </row>
-    <row r="26" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A26">
-        <v>12.5</v>
       </c>
       <c r="B26">
         <v>6.28</v>
       </c>
     </row>
-    <row r="27" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A27">
+        <v>12.5</v>
+      </c>
+      <c r="B27">
+        <v>6.28</v>
+      </c>
+    </row>
+    <row r="28" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A28">
         <v>13</v>
-      </c>
-      <c r="B27">
-        <v>6.33</v>
-      </c>
-    </row>
-    <row r="28" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A28">
-        <v>13.5</v>
       </c>
       <c r="B28">
         <v>6.33</v>
       </c>
     </row>
-    <row r="29" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A29">
+        <v>13.5</v>
+      </c>
+      <c r="B29">
+        <v>6.33</v>
+      </c>
+    </row>
+    <row r="30" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A30">
         <v>14</v>
-      </c>
-      <c r="B29">
-        <v>6.37</v>
-      </c>
-    </row>
-    <row r="30" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A30">
-        <v>14.5</v>
       </c>
       <c r="B30">
         <v>6.37</v>
       </c>
     </row>
-    <row r="31" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A31">
+        <v>14.5</v>
+      </c>
+      <c r="B31">
+        <v>6.37</v>
+      </c>
+    </row>
+    <row r="32" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A32">
         <v>15</v>
-      </c>
-      <c r="B31">
-        <v>6.41</v>
-      </c>
-    </row>
-    <row r="32" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A32">
-        <v>15.5</v>
       </c>
       <c r="B32">
         <v>6.41</v>
       </c>
     </row>
-    <row r="33" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A33">
+        <v>15.5</v>
+      </c>
+      <c r="B33">
+        <v>6.41</v>
+      </c>
+    </row>
+    <row r="34" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A34">
         <v>16</v>
-      </c>
-      <c r="B33">
-        <v>6.45</v>
-      </c>
-    </row>
-    <row r="34" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A34">
-        <v>16.5</v>
       </c>
       <c r="B34">
         <v>6.45</v>
       </c>
     </row>
-    <row r="35" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A35">
+        <v>16.5</v>
+      </c>
+      <c r="B35">
+        <v>6.45</v>
+      </c>
+    </row>
+    <row r="36" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A36">
         <v>17</v>
-      </c>
-      <c r="B35">
-        <v>6.48</v>
-      </c>
-    </row>
-    <row r="36" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A36">
-        <v>17.5</v>
       </c>
       <c r="B36">
         <v>6.48</v>
       </c>
     </row>
-    <row r="37" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="37" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A37">
+        <v>17.5</v>
+      </c>
+      <c r="B37">
+        <v>6.48</v>
+      </c>
+    </row>
+    <row r="38" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A38">
         <v>18</v>
-      </c>
-      <c r="B37">
-        <v>6.51</v>
-      </c>
-    </row>
-    <row r="38" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A38">
-        <v>18.5</v>
       </c>
       <c r="B38">
         <v>6.51</v>
       </c>
     </row>
-    <row r="39" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="39" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A39">
+        <v>18.5</v>
+      </c>
+      <c r="B39">
+        <v>6.51</v>
+      </c>
+    </row>
+    <row r="40" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A40">
         <v>19</v>
-      </c>
-      <c r="B39">
-        <v>6.54</v>
-      </c>
-    </row>
-    <row r="40" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A40">
-        <v>19.5</v>
       </c>
       <c r="B40">
         <v>6.54</v>
       </c>
     </row>
-    <row r="41" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="41" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A41">
+        <v>19.5</v>
+      </c>
+      <c r="B41">
+        <v>6.54</v>
+      </c>
+    </row>
+    <row r="42" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A42">
         <v>20</v>
       </c>
-      <c r="B41" s="1">
+      <c r="B42" s="1">
         <v>6.56</v>
       </c>
     </row>
-    <row r="42" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A42">
+    <row r="43" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A43">
         <v>20.5</v>
       </c>
-      <c r="B42">
+      <c r="B43">
         <v>6.56</v>
       </c>
     </row>
-    <row r="43" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A43">
+    <row r="44" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A44">
         <v>21</v>
-      </c>
-      <c r="B43">
-        <v>6.58</v>
-      </c>
-    </row>
-    <row r="44" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A44">
-        <v>21.5</v>
       </c>
       <c r="B44">
         <v>6.58</v>
       </c>
     </row>
-    <row r="45" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="45" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A45">
+        <v>21.5</v>
+      </c>
+      <c r="B45">
+        <v>6.58</v>
+      </c>
+    </row>
+    <row r="46" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A46">
         <v>22</v>
-      </c>
-      <c r="B45">
-        <v>6.6</v>
-      </c>
-    </row>
-    <row r="46" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A46">
-        <v>22.5</v>
       </c>
       <c r="B46">
         <v>6.6</v>
       </c>
     </row>
-    <row r="47" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="47" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A47">
+        <v>22.5</v>
+      </c>
+      <c r="B47">
+        <v>6.6</v>
+      </c>
+    </row>
+    <row r="48" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A48">
         <v>23</v>
-      </c>
-      <c r="B47">
-        <v>6.62</v>
-      </c>
-    </row>
-    <row r="48" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A48">
-        <v>23.5</v>
       </c>
       <c r="B48">
         <v>6.62</v>
       </c>
     </row>
-    <row r="49" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="49" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A49">
+        <v>23.5</v>
+      </c>
+      <c r="B49">
+        <v>6.62</v>
+      </c>
+    </row>
+    <row r="50" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A50">
         <v>24</v>
-      </c>
-      <c r="B49">
-        <v>6.63</v>
-      </c>
-    </row>
-    <row r="50" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A50">
-        <v>24.5</v>
       </c>
       <c r="B50">
         <v>6.63</v>
       </c>
     </row>
-    <row r="51" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="51" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A51">
+        <v>24.5</v>
+      </c>
+      <c r="B51">
+        <v>6.63</v>
+      </c>
+    </row>
+    <row r="52" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A52">
         <v>25</v>
-      </c>
-      <c r="B51">
-        <v>6.64</v>
-      </c>
-    </row>
-    <row r="52" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A52">
-        <v>25.5</v>
       </c>
       <c r="B52">
         <v>6.64</v>
       </c>
     </row>
-    <row r="53" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="53" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A53">
+        <v>25.5</v>
+      </c>
+      <c r="B53">
+        <v>6.64</v>
+      </c>
+    </row>
+    <row r="54" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A54">
         <v>26</v>
-      </c>
-      <c r="B53">
-        <v>6.66</v>
-      </c>
-    </row>
-    <row r="54" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A54">
-        <v>26.5</v>
       </c>
       <c r="B54">
         <v>6.66</v>
       </c>
     </row>
-    <row r="55" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="55" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A55">
+        <v>26.5</v>
+      </c>
+      <c r="B55">
+        <v>6.66</v>
+      </c>
+    </row>
+    <row r="56" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A56">
         <v>27</v>
-      </c>
-      <c r="B55">
-        <v>6.67</v>
-      </c>
-    </row>
-    <row r="56" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A56">
-        <v>27.5</v>
       </c>
       <c r="B56">
         <v>6.67</v>
       </c>
     </row>
-    <row r="57" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="57" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A57">
+        <v>27.5</v>
+      </c>
+      <c r="B57">
+        <v>6.67</v>
+      </c>
+    </row>
+    <row r="58" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A58">
         <v>28</v>
-      </c>
-      <c r="B57">
-        <v>6.68</v>
-      </c>
-    </row>
-    <row r="58" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A58">
-        <v>28.5</v>
       </c>
       <c r="B58">
         <v>6.68</v>
       </c>
     </row>
-    <row r="59" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="59" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A59">
-        <v>29</v>
+        <v>28.5</v>
       </c>
       <c r="B59">
         <v>6.68</v>
       </c>
     </row>
-    <row r="60" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="60" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A60">
-        <v>29.5</v>
+        <v>29</v>
       </c>
       <c r="B60">
         <v>6.68</v>
       </c>
     </row>
-    <row r="61" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="61" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A61">
+        <v>29.5</v>
+      </c>
+      <c r="B61">
+        <v>6.68</v>
+      </c>
+    </row>
+    <row r="62" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A62">
         <v>30</v>
       </c>
-      <c r="B61">
+      <c r="B62">
         <v>6.69</v>
       </c>
     </row>
-    <row r="62" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A62">
+    <row r="63" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A63">
         <v>30.5</v>
       </c>
-      <c r="B62">
+      <c r="B63">
         <v>6.69</v>
       </c>
     </row>

</xml_diff>